<commit_message>
updated printed parts guide images
</commit_message>
<xml_diff>
--- a/documentation/printed_parts_md_builder.xlsx
+++ b/documentation/printed_parts_md_builder.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f75adbc1b1328d64/Documents/GitHub/BabyBeltPro/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="125" documentId="8_{C0675C86-CF61-45B1-818F-376B7F2C33E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C70E4A89-FDA6-43EB-BD16-2A43B344F6C1}"/>
+  <xr:revisionPtr revIDLastSave="133" documentId="8_{C0675C86-CF61-45B1-818F-376B7F2C33E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{465D1310-E27D-4083-89B0-0385A64CF275}"/>
   <bookViews>
-    <workbookView xWindow="-42810" yWindow="3810" windowWidth="38700" windowHeight="15345" xr2:uid="{56CCDE47-8BF8-4249-AE9A-3862BA691127}"/>
+    <workbookView xWindow="-38205" yWindow="4965" windowWidth="19050" windowHeight="12435" xr2:uid="{56CCDE47-8BF8-4249-AE9A-3862BA691127}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$29</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="49">
   <si>
     <t>Name</t>
   </si>
@@ -161,9 +162,6 @@
     <t>./STLs/Gantry/Y/BBProV26fl_LinearRailReplacement.stl</t>
   </si>
   <si>
-    <t>./STLs/Gantry/Y/MMU &amp; AMS/TODO.txt</t>
-  </si>
-  <si>
     <t>./STLs/Gantry/Y/[a]_BBProV26fl_RockMonsterNo1YTentionerBody.stl</t>
   </si>
   <si>
@@ -186,6 +184,9 @@
   </si>
   <si>
     <t>./STLs/Gantry/X/[ai]_BBProV26fl_XrailMountUnder-SideB.stl</t>
+  </si>
+  <si>
+    <t>./STLs/Tools/[any]_BBPro_XRailSpacerV2[x2].stl</t>
   </si>
 </sst>
 </file>
@@ -558,7 +559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC80A11F-D4A9-4A4B-AA84-1AE963FFD50F}">
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="90.42578125" bestFit="1" customWidth="1"/>
@@ -599,7 +600,7 @@
         <v>3</v>
       </c>
       <c r="I1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J1" t="s">
         <v>7</v>
@@ -650,7 +651,7 @@
         <v>-----</v>
       </c>
       <c r="L2" t="str">
-        <f t="shared" ref="L2:L38" si="1">"|"&amp;$D2&amp;"|"&amp;$E2&amp;"|"&amp;$F2&amp;"|"&amp;$G2&amp;"|"&amp;$H2&amp;"|"&amp;$I2&amp;"|"&amp;$J2&amp;"|"&amp;$K2</f>
+        <f t="shared" ref="L2:L37" si="1">"|"&amp;$D2&amp;"|"&amp;$E2&amp;"|"&amp;$F2&amp;"|"&amp;$G2&amp;"|"&amp;$H2&amp;"|"&amp;$I2&amp;"|"&amp;$J2&amp;"|"&amp;$K2</f>
         <v>|-----|-----|-----|-----|-----|-----|-----|-----</v>
       </c>
     </row>
@@ -683,7 +684,7 @@
         <v>Main</v>
       </c>
       <c r="H3" t="str">
-        <f t="shared" ref="H3:H38" si="2">IF(_xlfn.REGEXTEST($B3,"\[\S*[s][^s\]]*\]"),"Yes","No")</f>
+        <f t="shared" ref="H3:H37" si="2">IF(_xlfn.REGEXTEST($B3,"\[\S*[s][^s\]]*\]"),"Yes","No")</f>
         <v>No</v>
       </c>
       <c r="I3" t="str">
@@ -691,7 +692,7 @@
         <v>No</v>
       </c>
       <c r="J3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L3" t="str">
         <f t="shared" si="1"/>
@@ -703,27 +704,27 @@
         <v>10</v>
       </c>
       <c r="B4" t="str">
-        <f t="shared" ref="B4:B38" si="3">_xlfn.TEXTAFTER($A4,"/",-1)</f>
+        <f t="shared" ref="B4:B37" si="3">_xlfn.TEXTAFTER($A4,"/",-1)</f>
         <v>BBProV25fl_Side-A.stl</v>
       </c>
       <c r="C4" t="str">
-        <f t="shared" ref="C4:C38" si="4">RIGHT(_xlfn.TEXTBEFORE($A4,"/",-1),LEN(_xlfn.TEXTBEFORE($A4,"/",-1))-7)</f>
+        <f t="shared" ref="C4:C37" si="4">RIGHT(_xlfn.TEXTBEFORE($A4,"/",-1),LEN(_xlfn.TEXTBEFORE($A4,"/",-1))-7)</f>
         <v>Frame</v>
       </c>
       <c r="D4" t="str">
-        <f t="shared" ref="D4:D38" si="5">"["&amp;LEFT($B4,LEN($B4)-4)&amp;"](../STLs/"&amp;SUBSTITUTE($C4," ","%20")&amp;"/"&amp;SUBSTITUTE($B4," ","%20")&amp;")"</f>
+        <f t="shared" ref="D4:D37" si="5">"["&amp;LEFT($B4,LEN($B4)-4)&amp;"](../STLs/"&amp;SUBSTITUTE($C4," ","%20")&amp;"/"&amp;SUBSTITUTE($B4," ","%20")&amp;")"</f>
         <v>[BBProV25fl_Side-A](../STLs/Frame/BBProV25fl_Side-A.stl)</v>
       </c>
       <c r="E4" t="str">
-        <f t="shared" ref="E4:E38" si="6">"!["&amp;LEFT($B4,LEN($B4)-4)&amp;"](./images/printed_parts/"&amp;SUBSTITUTE($C4," ","%20")&amp;"/"&amp;SUBSTITUTE(SUBSTITUTE($B4,".stl",".jpg")," ","%20")&amp;")"</f>
+        <f t="shared" ref="E4:E37" si="6">"!["&amp;LEFT($B4,LEN($B4)-4)&amp;"](./images/printed_parts/"&amp;SUBSTITUTE($C4," ","%20")&amp;"/"&amp;SUBSTITUTE(SUBSTITUTE($B4,".stl",".jpg")," ","%20")&amp;")"</f>
         <v>![BBProV25fl_Side-A](./images/printed_parts/Frame/BBProV25fl_Side-A.jpg)</v>
       </c>
       <c r="F4" t="str">
-        <f t="shared" ref="F4:F38" si="7">$C4</f>
+        <f t="shared" ref="F4:F37" si="7">$C4</f>
         <v>Frame</v>
       </c>
       <c r="G4" t="str">
-        <f t="shared" ref="G4:G38" si="8">IF(_xlfn.REGEXTEST($B4,"\[\S*[a][^a\]]*\]"),"Accent","Main")</f>
+        <f t="shared" ref="G4:G37" si="8">IF(_xlfn.REGEXTEST($B4,"\[\S*[a][^a\]]*\]"),"Accent","Main")</f>
         <v>Main</v>
       </c>
       <c r="H4" t="str">
@@ -731,11 +732,11 @@
         <v>No</v>
       </c>
       <c r="I4" t="str">
-        <f t="shared" ref="I4:I38" si="9">IF(_xlfn.REGEXTEST($B4,"\[\S*[i][^i\]]*\]"),"Yes","No")</f>
+        <f t="shared" ref="I4:I37" si="9">IF(_xlfn.REGEXTEST($B4,"\[\S*[i][^i\]]*\]"),"Yes","No")</f>
         <v>No</v>
       </c>
       <c r="J4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L4" t="str">
         <f t="shared" si="1"/>
@@ -779,7 +780,7 @@
         <v>No</v>
       </c>
       <c r="J5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L5" t="str">
         <f t="shared" si="1"/>
@@ -823,7 +824,7 @@
         <v>No</v>
       </c>
       <c r="J6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L6" t="str">
         <f t="shared" si="1"/>
@@ -867,7 +868,7 @@
         <v>No</v>
       </c>
       <c r="J7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L7" t="str">
         <f t="shared" si="1"/>
@@ -911,7 +912,7 @@
         <v>No</v>
       </c>
       <c r="J8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L8" t="str">
         <f t="shared" si="1"/>
@@ -955,7 +956,7 @@
         <v>No</v>
       </c>
       <c r="J9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L9" t="str">
         <f t="shared" si="1"/>
@@ -999,7 +1000,7 @@
         <v>No</v>
       </c>
       <c r="J10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L10" t="str">
         <f t="shared" si="1"/>
@@ -1043,7 +1044,7 @@
         <v>No</v>
       </c>
       <c r="J11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L11" t="str">
         <f t="shared" si="1"/>
@@ -1087,7 +1088,7 @@
         <v>No</v>
       </c>
       <c r="J12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L12" t="str">
         <f t="shared" si="1"/>
@@ -1131,7 +1132,7 @@
         <v>No</v>
       </c>
       <c r="J13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L13" t="str">
         <f t="shared" si="1"/>
@@ -1140,7 +1141,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="3"/>
@@ -1175,7 +1176,7 @@
         <v>Yes</v>
       </c>
       <c r="J14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L14" t="str">
         <f t="shared" si="1"/>
@@ -1219,7 +1220,7 @@
         <v>No</v>
       </c>
       <c r="J15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L15" t="str">
         <f t="shared" si="1"/>
@@ -1263,7 +1264,7 @@
         <v>No</v>
       </c>
       <c r="J16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L16" t="str">
         <f t="shared" si="1"/>
@@ -1307,7 +1308,7 @@
         <v>No</v>
       </c>
       <c r="J17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L17" t="str">
         <f t="shared" si="1"/>
@@ -1351,7 +1352,7 @@
         <v>No</v>
       </c>
       <c r="J18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L18" t="str">
         <f t="shared" si="1"/>
@@ -1395,7 +1396,7 @@
         <v>No</v>
       </c>
       <c r="J19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L19" t="str">
         <f t="shared" si="1"/>
@@ -1404,7 +1405,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="3"/>
@@ -1439,7 +1440,7 @@
         <v>Yes</v>
       </c>
       <c r="J20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L20" t="str">
         <f t="shared" si="1"/>
@@ -1448,7 +1449,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="3"/>
@@ -1483,7 +1484,7 @@
         <v>Yes</v>
       </c>
       <c r="J21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L21" t="str">
         <f t="shared" si="1"/>
@@ -1527,7 +1528,7 @@
         <v>No</v>
       </c>
       <c r="J22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L22" t="str">
         <f t="shared" si="1"/>
@@ -1571,7 +1572,7 @@
         <v>No</v>
       </c>
       <c r="J23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L23" t="str">
         <f t="shared" si="1"/>
@@ -1615,7 +1616,7 @@
         <v>No</v>
       </c>
       <c r="J24" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L24" t="str">
         <f t="shared" si="1"/>
@@ -1659,7 +1660,7 @@
         <v>No</v>
       </c>
       <c r="J25" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L25" t="str">
         <f t="shared" si="1"/>
@@ -1668,31 +1669,31 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="3"/>
-        <v>TODO.txt</v>
+        <v>[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder.stl</v>
       </c>
       <c r="C26" t="str">
         <f t="shared" si="4"/>
-        <v>Gantry/Y/MMU &amp; AMS</v>
+        <v>Gantry/Y</v>
       </c>
       <c r="D26" t="str">
         <f t="shared" si="5"/>
-        <v>[TODO](../STLs/Gantry/Y/MMU%20&amp;%20AMS/TODO.txt)</v>
+        <v>[[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder](../STLs/Gantry/Y/[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder.stl)</v>
       </c>
       <c r="E26" t="str">
         <f t="shared" si="6"/>
-        <v>![TODO](./images/printed_parts/Gantry/Y/MMU%20&amp;%20AMS/TODO.txt)</v>
+        <v>![[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder](./images/printed_parts/Gantry/Y/[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder.jpg)</v>
       </c>
       <c r="F26" t="str">
         <f t="shared" si="7"/>
-        <v>Gantry/Y/MMU &amp; AMS</v>
+        <v>Gantry/Y</v>
       </c>
       <c r="G26" t="str">
         <f t="shared" si="8"/>
-        <v>Main</v>
+        <v>Accent</v>
       </c>
       <c r="H26" t="str">
         <f t="shared" si="2"/>
@@ -1703,20 +1704,20 @@
         <v>No</v>
       </c>
       <c r="J26" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L26" t="str">
         <f t="shared" si="1"/>
-        <v>|[TODO](../STLs/Gantry/Y/MMU%20&amp;%20AMS/TODO.txt)|![TODO](./images/printed_parts/Gantry/Y/MMU%20&amp;%20AMS/TODO.txt)|Gantry/Y/MMU &amp; AMS|Main|No|No|&gt;= PLA|</v>
+        <v>|[[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder](../STLs/Gantry/Y/[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder.stl)|![[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder](./images/printed_parts/Gantry/Y/[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder.jpg)|Gantry/Y|Accent|No|No|&gt;= PLA|</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="3"/>
-        <v>[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder.stl</v>
+        <v>[a]_BBProV26fl_RockMonsterNo1YTentionerBody.stl</v>
       </c>
       <c r="C27" t="str">
         <f t="shared" si="4"/>
@@ -1724,11 +1725,11 @@
       </c>
       <c r="D27" t="str">
         <f t="shared" si="5"/>
-        <v>[[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder](../STLs/Gantry/Y/[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder.stl)</v>
+        <v>[[a]_BBProV26fl_RockMonsterNo1YTentionerBody](../STLs/Gantry/Y/[a]_BBProV26fl_RockMonsterNo1YTentionerBody.stl)</v>
       </c>
       <c r="E27" t="str">
         <f t="shared" si="6"/>
-        <v>![[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder](./images/printed_parts/Gantry/Y/[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder.jpg)</v>
+        <v>![[a]_BBProV26fl_RockMonsterNo1YTentionerBody](./images/printed_parts/Gantry/Y/[a]_BBProV26fl_RockMonsterNo1YTentionerBody.jpg)</v>
       </c>
       <c r="F27" t="str">
         <f t="shared" si="7"/>
@@ -1747,36 +1748,36 @@
         <v>No</v>
       </c>
       <c r="J27" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L27" t="str">
         <f t="shared" si="1"/>
-        <v>|[[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder](../STLs/Gantry/Y/[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder.stl)|![[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder](./images/printed_parts/Gantry/Y/[a]_BBProV25fl_RockMonsterNo1YTentionerIdlerHolder.jpg)|Gantry/Y|Accent|No|No|&gt;= PLA|</v>
+        <v>|[[a]_BBProV26fl_RockMonsterNo1YTentionerBody](../STLs/Gantry/Y/[a]_BBProV26fl_RockMonsterNo1YTentionerBody.stl)|![[a]_BBProV26fl_RockMonsterNo1YTentionerBody](./images/printed_parts/Gantry/Y/[a]_BBProV26fl_RockMonsterNo1YTentionerBody.jpg)|Gantry/Y|Accent|No|No|&gt;= PLA|</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="3"/>
-        <v>[a]_BBProV26fl_RockMonsterNo1YTentionerBody.stl</v>
+        <v>[a]_BBProV25fl_PrintBelt-Frame-A.stl</v>
       </c>
       <c r="C28" t="str">
         <f t="shared" si="4"/>
-        <v>Gantry/Y</v>
+        <v>PrintBelt</v>
       </c>
       <c r="D28" t="str">
         <f t="shared" si="5"/>
-        <v>[[a]_BBProV26fl_RockMonsterNo1YTentionerBody](../STLs/Gantry/Y/[a]_BBProV26fl_RockMonsterNo1YTentionerBody.stl)</v>
+        <v>[[a]_BBProV25fl_PrintBelt-Frame-A](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-A.stl)</v>
       </c>
       <c r="E28" t="str">
         <f t="shared" si="6"/>
-        <v>![[a]_BBProV26fl_RockMonsterNo1YTentionerBody](./images/printed_parts/Gantry/Y/[a]_BBProV26fl_RockMonsterNo1YTentionerBody.jpg)</v>
+        <v>![[a]_BBProV25fl_PrintBelt-Frame-A](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-A.jpg)</v>
       </c>
       <c r="F28" t="str">
         <f t="shared" si="7"/>
-        <v>Gantry/Y</v>
+        <v>PrintBelt</v>
       </c>
       <c r="G28" t="str">
         <f t="shared" si="8"/>
@@ -1791,20 +1792,20 @@
         <v>No</v>
       </c>
       <c r="J28" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L28" t="str">
         <f t="shared" si="1"/>
-        <v>|[[a]_BBProV26fl_RockMonsterNo1YTentionerBody](../STLs/Gantry/Y/[a]_BBProV26fl_RockMonsterNo1YTentionerBody.stl)|![[a]_BBProV26fl_RockMonsterNo1YTentionerBody](./images/printed_parts/Gantry/Y/[a]_BBProV26fl_RockMonsterNo1YTentionerBody.jpg)|Gantry/Y|Accent|No|No|&gt;= PLA|</v>
+        <v>|[[a]_BBProV25fl_PrintBelt-Frame-A](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-A.stl)|![[a]_BBProV25fl_PrintBelt-Frame-A](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-A.jpg)|PrintBelt|Accent|No|No|&gt;= PLA|</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="3"/>
-        <v>[a]_BBProV25fl_PrintBelt-Frame-A.stl</v>
+        <v>[a]_BBProV25fl_PrintBelt-Frame-B.stl</v>
       </c>
       <c r="C29" t="str">
         <f t="shared" si="4"/>
@@ -1812,11 +1813,11 @@
       </c>
       <c r="D29" t="str">
         <f t="shared" si="5"/>
-        <v>[[a]_BBProV25fl_PrintBelt-Frame-A](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-A.stl)</v>
+        <v>[[a]_BBProV25fl_PrintBelt-Frame-B](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-B.stl)</v>
       </c>
       <c r="E29" t="str">
         <f t="shared" si="6"/>
-        <v>![[a]_BBProV25fl_PrintBelt-Frame-A](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-A.jpg)</v>
+        <v>![[a]_BBProV25fl_PrintBelt-Frame-B](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-B.jpg)</v>
       </c>
       <c r="F29" t="str">
         <f t="shared" si="7"/>
@@ -1835,20 +1836,20 @@
         <v>No</v>
       </c>
       <c r="J29" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L29" t="str">
         <f t="shared" si="1"/>
-        <v>|[[a]_BBProV25fl_PrintBelt-Frame-A](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-A.stl)|![[a]_BBProV25fl_PrintBelt-Frame-A](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-A.jpg)|PrintBelt|Accent|No|No|&gt;= PLA|</v>
+        <v>|[[a]_BBProV25fl_PrintBelt-Frame-B](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-B.stl)|![[a]_BBProV25fl_PrintBelt-Frame-B](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-B.jpg)|PrintBelt|Accent|No|No|&gt;= PLA|</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="3"/>
-        <v>[a]_BBProV25fl_PrintBelt-Frame-B.stl</v>
+        <v>[a]_BBProV25fl_PrintBelt-Nut(2x).stl</v>
       </c>
       <c r="C30" t="str">
         <f t="shared" si="4"/>
@@ -1856,11 +1857,11 @@
       </c>
       <c r="D30" t="str">
         <f t="shared" si="5"/>
-        <v>[[a]_BBProV25fl_PrintBelt-Frame-B](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-B.stl)</v>
+        <v>[[a]_BBProV25fl_PrintBelt-Nut(2x)](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Nut(2x).stl)</v>
       </c>
       <c r="E30" t="str">
         <f t="shared" si="6"/>
-        <v>![[a]_BBProV25fl_PrintBelt-Frame-B](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-B.jpg)</v>
+        <v>![[a]_BBProV25fl_PrintBelt-Nut(2x)](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Nut(2x).jpg)</v>
       </c>
       <c r="F30" t="str">
         <f t="shared" si="7"/>
@@ -1879,20 +1880,20 @@
         <v>No</v>
       </c>
       <c r="J30" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L30" t="str">
         <f t="shared" si="1"/>
-        <v>|[[a]_BBProV25fl_PrintBelt-Frame-B](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-B.stl)|![[a]_BBProV25fl_PrintBelt-Frame-B](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Frame-B.jpg)|PrintBelt|Accent|No|No|&gt;= PLA|</v>
+        <v>|[[a]_BBProV25fl_PrintBelt-Nut(2x)](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Nut(2x).stl)|![[a]_BBProV25fl_PrintBelt-Nut(2x)](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Nut(2x).jpg)|PrintBelt|Accent|No|No|&gt;= PLA|</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="3"/>
-        <v>[a]_BBProV25fl_PrintBelt-Nut(2x).stl</v>
+        <v>[a]_BBProV25fl_PrintBelt-Pusher-A.stl</v>
       </c>
       <c r="C31" t="str">
         <f t="shared" si="4"/>
@@ -1900,11 +1901,11 @@
       </c>
       <c r="D31" t="str">
         <f t="shared" si="5"/>
-        <v>[[a]_BBProV25fl_PrintBelt-Nut(2x)](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Nut(2x).stl)</v>
+        <v>[[a]_BBProV25fl_PrintBelt-Pusher-A](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-A.stl)</v>
       </c>
       <c r="E31" t="str">
         <f t="shared" si="6"/>
-        <v>![[a]_BBProV25fl_PrintBelt-Nut(2x)](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Nut(2x).jpg)</v>
+        <v>![[a]_BBProV25fl_PrintBelt-Pusher-A](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-A.jpg)</v>
       </c>
       <c r="F31" t="str">
         <f t="shared" si="7"/>
@@ -1923,20 +1924,20 @@
         <v>No</v>
       </c>
       <c r="J31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L31" t="str">
         <f t="shared" si="1"/>
-        <v>|[[a]_BBProV25fl_PrintBelt-Nut(2x)](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Nut(2x).stl)|![[a]_BBProV25fl_PrintBelt-Nut(2x)](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Nut(2x).jpg)|PrintBelt|Accent|No|No|&gt;= PLA|</v>
+        <v>|[[a]_BBProV25fl_PrintBelt-Pusher-A](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-A.stl)|![[a]_BBProV25fl_PrintBelt-Pusher-A](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-A.jpg)|PrintBelt|Accent|No|No|&gt;= PLA|</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="3"/>
-        <v>[a]_BBProV25fl_PrintBelt-Pusher-A.stl</v>
+        <v>[a]_BBProV25fl_PrintBelt-Pusher-B.stl</v>
       </c>
       <c r="C32" t="str">
         <f t="shared" si="4"/>
@@ -1944,11 +1945,11 @@
       </c>
       <c r="D32" t="str">
         <f t="shared" si="5"/>
-        <v>[[a]_BBProV25fl_PrintBelt-Pusher-A](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-A.stl)</v>
+        <v>[[a]_BBProV25fl_PrintBelt-Pusher-B](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-B.stl)</v>
       </c>
       <c r="E32" t="str">
         <f t="shared" si="6"/>
-        <v>![[a]_BBProV25fl_PrintBelt-Pusher-A](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-A.jpg)</v>
+        <v>![[a]_BBProV25fl_PrintBelt-Pusher-B](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-B.jpg)</v>
       </c>
       <c r="F32" t="str">
         <f t="shared" si="7"/>
@@ -1967,36 +1968,36 @@
         <v>No</v>
       </c>
       <c r="J32" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L32" t="str">
         <f t="shared" si="1"/>
-        <v>|[[a]_BBProV25fl_PrintBelt-Pusher-A](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-A.stl)|![[a]_BBProV25fl_PrintBelt-Pusher-A](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-A.jpg)|PrintBelt|Accent|No|No|&gt;= PLA|</v>
+        <v>|[[a]_BBProV25fl_PrintBelt-Pusher-B](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-B.stl)|![[a]_BBProV25fl_PrintBelt-Pusher-B](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-B.jpg)|PrintBelt|Accent|No|No|&gt;= PLA|</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="3"/>
-        <v>[a]_BBProV25fl_PrintBelt-Pusher-B.stl</v>
+        <v>[a,s]_BBProV25fl_Roller[x2].stl</v>
       </c>
       <c r="C33" t="str">
         <f t="shared" si="4"/>
-        <v>PrintBelt</v>
+        <v>ZBeltDrive</v>
       </c>
       <c r="D33" t="str">
         <f t="shared" si="5"/>
-        <v>[[a]_BBProV25fl_PrintBelt-Pusher-B](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-B.stl)</v>
+        <v>[[a,s]_BBProV25fl_Roller[x2]](../STLs/ZBeltDrive/[a,s]_BBProV25fl_Roller[x2].stl)</v>
       </c>
       <c r="E33" t="str">
         <f t="shared" si="6"/>
-        <v>![[a]_BBProV25fl_PrintBelt-Pusher-B](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-B.jpg)</v>
+        <v>![[a,s]_BBProV25fl_Roller[x2]](./images/printed_parts/ZBeltDrive/[a,s]_BBProV25fl_Roller[x2].jpg)</v>
       </c>
       <c r="F33" t="str">
         <f t="shared" si="7"/>
-        <v>PrintBelt</v>
+        <v>ZBeltDrive</v>
       </c>
       <c r="G33" t="str">
         <f t="shared" si="8"/>
@@ -2004,27 +2005,27 @@
       </c>
       <c r="H33" t="str">
         <f t="shared" si="2"/>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="I33" t="str">
         <f t="shared" si="9"/>
         <v>No</v>
       </c>
       <c r="J33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L33" t="str">
         <f t="shared" si="1"/>
-        <v>|[[a]_BBProV25fl_PrintBelt-Pusher-B](../STLs/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-B.stl)|![[a]_BBProV25fl_PrintBelt-Pusher-B](./images/printed_parts/PrintBelt/[a]_BBProV25fl_PrintBelt-Pusher-B.jpg)|PrintBelt|Accent|No|No|&gt;= PLA|</v>
+        <v>|[[a,s]_BBProV25fl_Roller[x2]](../STLs/ZBeltDrive/[a,s]_BBProV25fl_Roller[x2].stl)|![[a,s]_BBProV25fl_Roller[x2]](./images/printed_parts/ZBeltDrive/[a,s]_BBProV25fl_Roller[x2].jpg)|ZBeltDrive|Accent|Yes|No|&gt;= PLA|</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="3"/>
-        <v>[a,s]_BBProV25fl_Roller[x2].stl</v>
+        <v>[a]_BBProV25fl_Nema17_ZGear.stl</v>
       </c>
       <c r="C34" t="str">
         <f t="shared" si="4"/>
@@ -2032,11 +2033,11 @@
       </c>
       <c r="D34" t="str">
         <f t="shared" si="5"/>
-        <v>[[a,s]_BBProV25fl_Roller[x2]](../STLs/ZBeltDrive/[a,s]_BBProV25fl_Roller[x2].stl)</v>
+        <v>[[a]_BBProV25fl_Nema17_ZGear](../STLs/ZBeltDrive/[a]_BBProV25fl_Nema17_ZGear.stl)</v>
       </c>
       <c r="E34" t="str">
         <f t="shared" si="6"/>
-        <v>![[a,s]_BBProV25fl_Roller[x2]](./images/printed_parts/ZBeltDrive/[a,s]_BBProV25fl_Roller[x2].jpg)</v>
+        <v>![[a]_BBProV25fl_Nema17_ZGear](./images/printed_parts/ZBeltDrive/[a]_BBProV25fl_Nema17_ZGear.jpg)</v>
       </c>
       <c r="F34" t="str">
         <f t="shared" si="7"/>
@@ -2048,7 +2049,7 @@
       </c>
       <c r="H34" t="str">
         <f t="shared" si="2"/>
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="I34" t="str">
         <f t="shared" si="9"/>
@@ -2059,16 +2060,16 @@
       </c>
       <c r="L34" t="str">
         <f t="shared" si="1"/>
-        <v>|[[a,s]_BBProV25fl_Roller[x2]](../STLs/ZBeltDrive/[a,s]_BBProV25fl_Roller[x2].stl)|![[a,s]_BBProV25fl_Roller[x2]](./images/printed_parts/ZBeltDrive/[a,s]_BBProV25fl_Roller[x2].jpg)|ZBeltDrive|Accent|Yes|No|&gt;= PLA|</v>
+        <v>|[[a]_BBProV25fl_Nema17_ZGear](../STLs/ZBeltDrive/[a]_BBProV25fl_Nema17_ZGear.stl)|![[a]_BBProV25fl_Nema17_ZGear](./images/printed_parts/ZBeltDrive/[a]_BBProV25fl_Nema17_ZGear.jpg)|ZBeltDrive|Accent|No|No|&gt;= PETG|</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="3"/>
-        <v>[a]_BBProV25fl_Nema17_ZGear.stl</v>
+        <v>[a]_BBProV25fl_Roller_ZGear.stl</v>
       </c>
       <c r="C35" t="str">
         <f t="shared" si="4"/>
@@ -2076,11 +2077,11 @@
       </c>
       <c r="D35" t="str">
         <f t="shared" si="5"/>
-        <v>[[a]_BBProV25fl_Nema17_ZGear](../STLs/ZBeltDrive/[a]_BBProV25fl_Nema17_ZGear.stl)</v>
+        <v>[[a]_BBProV25fl_Roller_ZGear](../STLs/ZBeltDrive/[a]_BBProV25fl_Roller_ZGear.stl)</v>
       </c>
       <c r="E35" t="str">
         <f t="shared" si="6"/>
-        <v>![[a]_BBProV25fl_Nema17_ZGear](./images/printed_parts/ZBeltDrive/[a]_BBProV25fl_Nema17_ZGear.jpg)</v>
+        <v>![[a]_BBProV25fl_Roller_ZGear](./images/printed_parts/ZBeltDrive/[a]_BBProV25fl_Roller_ZGear.jpg)</v>
       </c>
       <c r="F35" t="str">
         <f t="shared" si="7"/>
@@ -2099,20 +2100,20 @@
         <v>No</v>
       </c>
       <c r="J35" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L35" t="str">
         <f t="shared" si="1"/>
-        <v>|[[a]_BBProV25fl_Nema17_ZGear](../STLs/ZBeltDrive/[a]_BBProV25fl_Nema17_ZGear.stl)|![[a]_BBProV25fl_Nema17_ZGear](./images/printed_parts/ZBeltDrive/[a]_BBProV25fl_Nema17_ZGear.jpg)|ZBeltDrive|Accent|No|No|&gt;= PETG|</v>
+        <v>|[[a]_BBProV25fl_Roller_ZGear](../STLs/ZBeltDrive/[a]_BBProV25fl_Roller_ZGear.stl)|![[a]_BBProV25fl_Roller_ZGear](./images/printed_parts/ZBeltDrive/[a]_BBProV25fl_Roller_ZGear.jpg)|ZBeltDrive|Accent|No|No|&gt;= PETG|</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="3"/>
-        <v>[a]_BBProV25fl_Roller_ZGear.stl</v>
+        <v>[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED.stl</v>
       </c>
       <c r="C36" t="str">
         <f t="shared" si="4"/>
@@ -2120,11 +2121,11 @@
       </c>
       <c r="D36" t="str">
         <f t="shared" si="5"/>
-        <v>[[a]_BBProV25fl_Roller_ZGear](../STLs/ZBeltDrive/[a]_BBProV25fl_Roller_ZGear.stl)</v>
+        <v>[[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED](../STLs/ZBeltDrive/[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED.stl)</v>
       </c>
       <c r="E36" t="str">
         <f t="shared" si="6"/>
-        <v>![[a]_BBProV25fl_Roller_ZGear](./images/printed_parts/ZBeltDrive/[a]_BBProV25fl_Roller_ZGear.jpg)</v>
+        <v>![[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED](./images/printed_parts/ZBeltDrive/[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED.jpg)</v>
       </c>
       <c r="F36" t="str">
         <f t="shared" si="7"/>
@@ -2132,7 +2133,7 @@
       </c>
       <c r="G36" t="str">
         <f t="shared" si="8"/>
-        <v>Accent</v>
+        <v>Main</v>
       </c>
       <c r="H36" t="str">
         <f t="shared" si="2"/>
@@ -2143,20 +2144,20 @@
         <v>No</v>
       </c>
       <c r="J36" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L36" t="str">
         <f t="shared" si="1"/>
-        <v>|[[a]_BBProV25fl_Roller_ZGear](../STLs/ZBeltDrive/[a]_BBProV25fl_Roller_ZGear.stl)|![[a]_BBProV25fl_Roller_ZGear](./images/printed_parts/ZBeltDrive/[a]_BBProV25fl_Roller_ZGear.jpg)|ZBeltDrive|Accent|No|No|&gt;= PETG|</v>
+        <v>|[[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED](../STLs/ZBeltDrive/[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED.stl)|![[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED](./images/printed_parts/ZBeltDrive/[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED.jpg)|ZBeltDrive|Main|No|No|&gt;= PETG|</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="3"/>
-        <v>[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED.stl</v>
+        <v>[HT]_BBProV25fl_UnderbedOrBed.stl</v>
       </c>
       <c r="C37" t="str">
         <f t="shared" si="4"/>
@@ -2164,11 +2165,11 @@
       </c>
       <c r="D37" t="str">
         <f t="shared" si="5"/>
-        <v>[[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED](../STLs/ZBeltDrive/[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED.stl)</v>
+        <v>[[HT]_BBProV25fl_UnderbedOrBed](../STLs/ZBeltDrive/[HT]_BBProV25fl_UnderbedOrBed.stl)</v>
       </c>
       <c r="E37" t="str">
         <f t="shared" si="6"/>
-        <v>![[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED](./images/printed_parts/ZBeltDrive/[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED.jpg)</v>
+        <v>![[HT]_BBProV25fl_UnderbedOrBed](./images/printed_parts/ZBeltDrive/[HT]_BBProV25fl_UnderbedOrBed.jpg)</v>
       </c>
       <c r="F37" t="str">
         <f t="shared" si="7"/>
@@ -2187,60 +2188,206 @@
         <v>No</v>
       </c>
       <c r="J37" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L37" t="str">
         <f t="shared" si="1"/>
-        <v>|[[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED](../STLs/ZBeltDrive/[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED.stl)|![[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED](./images/printed_parts/ZBeltDrive/[HT]_BBProV25fl_Underbed-notforbed-FOR_LDO_HEATBED.jpg)|ZBeltDrive|Main|No|No|&gt;= PETG|</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>30</v>
-      </c>
-      <c r="B38" t="str">
-        <f t="shared" si="3"/>
-        <v>[HT]_BBProV25fl_UnderbedOrBed.stl</v>
-      </c>
-      <c r="C38" t="str">
-        <f t="shared" si="4"/>
-        <v>ZBeltDrive</v>
-      </c>
-      <c r="D38" t="str">
-        <f t="shared" si="5"/>
-        <v>[[HT]_BBProV25fl_UnderbedOrBed](../STLs/ZBeltDrive/[HT]_BBProV25fl_UnderbedOrBed.stl)</v>
-      </c>
-      <c r="E38" t="str">
-        <f t="shared" si="6"/>
-        <v>![[HT]_BBProV25fl_UnderbedOrBed](./images/printed_parts/ZBeltDrive/[HT]_BBProV25fl_UnderbedOrBed.jpg)</v>
-      </c>
-      <c r="F38" t="str">
-        <f t="shared" si="7"/>
-        <v>ZBeltDrive</v>
-      </c>
-      <c r="G38" t="str">
-        <f t="shared" si="8"/>
-        <v>Main</v>
-      </c>
-      <c r="H38" t="str">
-        <f t="shared" si="2"/>
-        <v>No</v>
-      </c>
-      <c r="I38" t="str">
-        <f t="shared" si="9"/>
-        <v>No</v>
-      </c>
-      <c r="J38" t="s">
-        <v>44</v>
-      </c>
-      <c r="L38" t="str">
-        <f t="shared" si="1"/>
         <v>|[[HT]_BBProV25fl_UnderbedOrBed](../STLs/ZBeltDrive/[HT]_BBProV25fl_UnderbedOrBed.stl)|![[HT]_BBProV25fl_UnderbedOrBed](./images/printed_parts/ZBeltDrive/[HT]_BBProV25fl_UnderbedOrBed.jpg)|ZBeltDrive|Main|No|No|&gt;= PETG|</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L30" xr:uid="{CC80A11F-D4A9-4A4B-AA84-1AE963FFD50F}"/>
+  <autoFilter ref="A1:L29" xr:uid="{CC80A11F-D4A9-4A4B-AA84-1AE963FFD50F}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D456E13-C026-4130-A0C7-EBCEAF50CBC3}">
+  <dimension ref="A1:A36"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>